<commit_message>
Update cpl and bom
</commit_message>
<xml_diff>
--- a/Manufacturing/cpl.xlsx
+++ b/Manufacturing/cpl.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\Downloads\inktime\Manufacturing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D71EE9-1C48-457E-A232-D3D144B165BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0900C116-AC5E-458A-9C7C-978E3F5B9FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="3255" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="92">
   <si>
     <t>Designator</t>
   </si>
@@ -295,6 +295,12 @@
   </si>
   <si>
     <t>X2</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R4</t>
   </si>
 </sst>
 </file>
@@ -366,7 +372,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -376,6 +382,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -651,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
@@ -1749,7 +1756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:8">
       <c r="A65" s="2" t="s">
         <v>70</v>
       </c>
@@ -1766,7 +1773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:8">
       <c r="A66" s="2" t="s">
         <v>71</v>
       </c>
@@ -1783,7 +1790,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:8">
       <c r="A67" s="2" t="s">
         <v>72</v>
       </c>
@@ -1800,7 +1807,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:8">
       <c r="A68" s="2" t="s">
         <v>73</v>
       </c>
@@ -1817,7 +1824,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:8">
       <c r="A69" s="2" t="s">
         <v>74</v>
       </c>
@@ -1834,97 +1841,100 @@
         <v>180</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:8">
       <c r="A70" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B70" s="2">
+        <v>-11.3</v>
+      </c>
+      <c r="C70" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E70" s="2">
+        <v>90</v>
+      </c>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B71" s="2">
         <v>-6.1</v>
       </c>
-      <c r="C70" s="2">
+      <c r="C71" s="2">
         <v>7.8</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E70" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5">
-      <c r="A71" s="2" t="s">
+      <c r="D71" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E71" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B72" s="2">
         <v>-1.75</v>
       </c>
-      <c r="C71" s="2">
+      <c r="C72" s="2">
         <v>10.199999999999999</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E71" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5">
-      <c r="A72" s="2" t="s">
+      <c r="D72" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E72" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B73" s="2">
         <v>6</v>
       </c>
-      <c r="C72" s="2">
+      <c r="C73" s="2">
         <v>-9.9</v>
       </c>
-      <c r="D72" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E72" s="2">
+      <c r="D73" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E73" s="2">
         <v>270</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
-      <c r="A73" s="2" t="s">
+    <row r="74" spans="1:8" s="3" customFormat="1">
+      <c r="A74" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B74" s="2">
+        <v>-9.1</v>
+      </c>
+      <c r="C74" s="2">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E74" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B73" s="2">
+      <c r="B75" s="2">
         <v>-14.7</v>
-      </c>
-      <c r="C73" s="2">
-        <v>-14.4</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E73" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5">
-      <c r="A74" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B74" s="2">
-        <v>7.1</v>
-      </c>
-      <c r="C74" s="2">
-        <v>-14.4</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E74" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5">
-      <c r="A75" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B75" s="2">
-        <v>-3.7</v>
       </c>
       <c r="C75" s="2">
         <v>-14.4</v>
@@ -1936,97 +1946,97 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:8">
       <c r="A76" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B76" s="2">
+        <v>7.1</v>
+      </c>
+      <c r="C76" s="2">
+        <v>-14.4</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E76" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B77" s="2">
+        <v>-3.7</v>
+      </c>
+      <c r="C77" s="2">
+        <v>-14.4</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E77" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B76" s="2">
+      <c r="B78" s="2">
         <v>19.3</v>
       </c>
-      <c r="C76" s="2">
+      <c r="C78" s="2">
         <v>12.1</v>
       </c>
-      <c r="D76" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E76" s="2">
+      <c r="D78" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E78" s="2">
         <v>90</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
-      <c r="A77" s="2" t="s">
+    <row r="79" spans="1:8">
+      <c r="A79" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B77" s="2">
+      <c r="B79" s="2">
         <v>-6.4</v>
       </c>
-      <c r="C77" s="2">
+      <c r="C79" s="2">
         <v>-2.6</v>
       </c>
-      <c r="D77" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E77" s="2">
+      <c r="D79" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E79" s="2">
         <v>90</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
-      <c r="A78" s="2" t="s">
+    <row r="80" spans="1:8">
+      <c r="A80" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B78" s="2">
+      <c r="B80" s="2">
         <v>-7</v>
       </c>
-      <c r="C78" s="2">
+      <c r="C80" s="2">
         <v>5.85</v>
       </c>
-      <c r="D78" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E78" s="2">
+      <c r="D80" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E80" s="2">
         <v>270</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5">
-      <c r="A79" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B79" s="2">
-        <v>11</v>
-      </c>
-      <c r="C79" s="2">
-        <v>-13.83</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E79" s="2">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5">
-      <c r="A80" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B80" s="2">
-        <v>0</v>
-      </c>
-      <c r="C80" s="2">
-        <v>-13.83</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E80" s="2">
-        <v>180</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B81" s="2">
-        <v>-11</v>
+        <v>11</v>
       </c>
       <c r="C81" s="2">
         <v>-13.83</v>
@@ -2040,69 +2050,103 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" s="2" t="s">
-        <v>8</v>
+        <v>85</v>
       </c>
       <c r="B82" s="2">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="C82" s="2">
-        <v>-5.4</v>
+        <v>-13.83</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E82" s="2">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B83" s="2">
-        <v>18</v>
+        <v>-11</v>
       </c>
       <c r="C83" s="2">
-        <v>6.5</v>
+        <v>-13.83</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E83" s="2">
-        <v>270</v>
+        <v>180</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" s="2" t="s">
-        <v>88</v>
+        <v>8</v>
       </c>
       <c r="B84" s="2">
-        <v>16.5</v>
+        <v>12.5</v>
       </c>
       <c r="C84" s="2">
-        <v>-0.3</v>
+        <v>-5.4</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E84" s="2">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:5">
       <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="2">
+        <v>18</v>
+      </c>
+      <c r="C85" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E85" s="2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="2">
+        <v>16.5</v>
+      </c>
+      <c r="C86" s="2">
+        <v>-0.3</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E86" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B85" s="2">
+      <c r="B87" s="2">
         <v>6.8</v>
       </c>
-      <c r="C85" s="2">
+      <c r="C87" s="2">
         <v>-3.5</v>
       </c>
-      <c r="D85" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E85" s="2">
+      <c r="D87" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E87" s="2">
         <v>270</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use the correct library component for the 0201/0402 capacitors
</commit_message>
<xml_diff>
--- a/Manufacturing/cpl.xlsx
+++ b/Manufacturing/cpl.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\Downloads\inktime\Manufacturing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0900C116-AC5E-458A-9C7C-978E3F5B9FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4650353C-CBB2-4728-BBE9-BBCB284EF767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -707,10 +707,10 @@
         <v>5</v>
       </c>
       <c r="B3" s="2">
-        <v>16.649999999999999</v>
+        <v>16.75</v>
       </c>
       <c r="C3" s="2">
-        <v>-2.2000000000000002</v>
+        <v>-2</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
@@ -741,10 +741,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="2">
-        <v>16.649999999999999</v>
+        <v>16.75</v>
       </c>
       <c r="C5" s="2">
-        <v>-3</v>
+        <v>-2.8</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>10</v>
@@ -758,10 +758,10 @@
         <v>13</v>
       </c>
       <c r="B6" s="2">
-        <v>14.6</v>
+        <v>14.7</v>
       </c>
       <c r="C6" s="2">
-        <v>-1</v>
+        <v>-0.98</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -795,7 +795,7 @@
         <v>12.5</v>
       </c>
       <c r="C8" s="2">
-        <v>0.35</v>
+        <v>0.65</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
@@ -809,10 +809,10 @@
         <v>16</v>
       </c>
       <c r="B9" s="2">
-        <v>12</v>
+        <v>12.18</v>
       </c>
       <c r="C9" s="2">
-        <v>-0.55000000000000004</v>
+        <v>-0.27</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -829,7 +829,7 @@
         <v>5.2</v>
       </c>
       <c r="C10" s="2">
-        <v>-2.5</v>
+        <v>-2.75</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -846,7 +846,7 @@
         <v>5.2</v>
       </c>
       <c r="C11" s="2">
-        <v>-4.5</v>
+        <v>-4.3499999999999996</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -945,10 +945,10 @@
         <v>23</v>
       </c>
       <c r="B17" s="2">
-        <v>-5.9</v>
+        <v>-5.8</v>
       </c>
       <c r="C17" s="2">
-        <v>13</v>
+        <v>13.27</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -962,10 +962,10 @@
         <v>24</v>
       </c>
       <c r="B18" s="2">
-        <v>-5.9</v>
+        <v>-5.79</v>
       </c>
       <c r="C18" s="2">
-        <v>14.6</v>
+        <v>15.28</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -996,10 +996,10 @@
         <v>26</v>
       </c>
       <c r="B20" s="2">
-        <v>17.399999999999999</v>
+        <v>17.2</v>
       </c>
       <c r="C20" s="2">
-        <v>9.1</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
@@ -1030,7 +1030,7 @@
         <v>7</v>
       </c>
       <c r="B22" s="2">
-        <v>17.82</v>
+        <v>17.7</v>
       </c>
       <c r="C22" s="2">
         <v>-8.6999999999999993</v>
@@ -1115,10 +1115,10 @@
         <v>32</v>
       </c>
       <c r="B27" s="2">
-        <v>-17.7</v>
+        <v>-17.399999999999999</v>
       </c>
       <c r="C27" s="2">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>10</v>
@@ -1183,7 +1183,7 @@
         <v>36</v>
       </c>
       <c r="B31" s="2">
-        <v>17.82</v>
+        <v>17.7</v>
       </c>
       <c r="C31" s="2">
         <v>-9.5</v>
@@ -1200,16 +1200,16 @@
         <v>37</v>
       </c>
       <c r="B32" s="2">
-        <v>3</v>
+        <v>5.45</v>
       </c>
       <c r="C32" s="2">
-        <v>10</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E32" s="2">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -1217,16 +1217,16 @@
         <v>38</v>
       </c>
       <c r="B33" s="2">
-        <v>4.5999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="C33" s="2">
-        <v>8.6999999999999993</v>
+        <v>9.58</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E33" s="2">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -1268,7 +1268,7 @@
         <v>41</v>
       </c>
       <c r="B36" s="2">
-        <v>12.75</v>
+        <v>12.85</v>
       </c>
       <c r="C36" s="2">
         <v>-10.050000000000001</v>
@@ -1285,10 +1285,10 @@
         <v>42</v>
       </c>
       <c r="B37" s="2">
-        <v>16.5</v>
+        <v>16.2</v>
       </c>
       <c r="C37" s="2">
-        <v>-9</v>
+        <v>-8.8000000000000007</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>10</v>
@@ -2124,7 +2124,7 @@
         <v>16.5</v>
       </c>
       <c r="C86" s="2">
-        <v>-0.3</v>
+        <v>-0.1</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>10</v>

</xml_diff>